<commit_message>
new cricket stats updated
</commit_message>
<xml_diff>
--- a/cricket_stats.xlsx
+++ b/cricket_stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Desktop\MY UI's\cricket_streamlit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D48F000-E6B4-4CFB-9060-7F2017EF2731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5AC404C-7149-46FE-9A9F-F9A55E3F45D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="61">
   <si>
     <t>Date</t>
   </si>
@@ -203,6 +203,9 @@
   </si>
   <si>
     <t>Bohras CC</t>
+  </si>
+  <si>
+    <t>NCC (div 3)</t>
   </si>
 </sst>
 </file>
@@ -556,7 +559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P41"/>
+  <dimension ref="A1:P46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2059,6 +2062,70 @@
         <v>40</v>
       </c>
     </row>
+    <row r="42" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B42">
+        <v>2026</v>
+      </c>
+      <c r="C42" t="s">
+        <v>60</v>
+      </c>
+      <c r="D42" t="s">
+        <v>35</v>
+      </c>
+      <c r="E42">
+        <v>5</v>
+      </c>
+      <c r="F42">
+        <v>28</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
+      </c>
+      <c r="I42" t="s">
+        <v>38</v>
+      </c>
+      <c r="K42">
+        <v>1</v>
+      </c>
+      <c r="L42">
+        <v>6</v>
+      </c>
+      <c r="M42">
+        <v>39</v>
+      </c>
+      <c r="N42">
+        <v>1</v>
+      </c>
+      <c r="O42">
+        <v>1</v>
+      </c>
+      <c r="P42">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B43">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="44" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B44">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="45" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B45">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="46" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B46">
+        <v>2026</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:P40" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>